<commit_message>
Update with new samples
</commit_message>
<xml_diff>
--- a/feat_table.xlsx
+++ b/feat_table.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10419"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10426"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://o365coloradoedu-my.sharepoint.com/personal/ivta1597_colorado_edu/Documents/Shirts Lab/LCA_boltz_models/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="251" documentId="8_{C6F54AFA-60FD-B04F-BBB7-75B2589805D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{98C81B9C-A214-B645-BBD6-D23916481040}"/>
+  <xr:revisionPtr revIDLastSave="275" documentId="8_{C6F54AFA-60FD-B04F-BBB7-75B2589805D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6745F076-15FE-074D-A0B3-36934448A97A}"/>
   <bookViews>
-    <workbookView xWindow="41020" yWindow="3760" windowWidth="29400" windowHeight="17160" activeTab="1" xr2:uid="{27E63E85-0623-8743-9D49-3663B37B390F}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" activeTab="1" xr2:uid="{27E63E85-0623-8743-9D49-3663B37B390F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="227" uniqueCount="51">
   <si>
     <t>Group</t>
   </si>
@@ -166,6 +166,33 @@
   </si>
   <si>
     <t>0272</t>
+  </si>
+  <si>
+    <t>0246</t>
+  </si>
+  <si>
+    <t>0065</t>
+  </si>
+  <si>
+    <t>0947</t>
+  </si>
+  <si>
+    <t>0948</t>
+  </si>
+  <si>
+    <t>1413</t>
+  </si>
+  <si>
+    <t>0263</t>
+  </si>
+  <si>
+    <t>0540</t>
+  </si>
+  <si>
+    <t>0997</t>
+  </si>
+  <si>
+    <t>1745</t>
   </si>
 </sst>
 </file>
@@ -655,7 +682,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E67669D-DCA0-184E-97A6-09176FE4B22E}">
-  <dimension ref="A1:V85"/>
+  <dimension ref="A1:V82"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="11"/>
@@ -788,7 +815,7 @@
         <v>12</v>
       </c>
       <c r="C3" s="7">
-        <f t="shared" ref="C3:C64" si="0">IF(B3="Binder", 1,0)</f>
+        <f t="shared" ref="C3:C66" si="0">IF(B3="Binder", 1,0)</f>
         <v>1</v>
       </c>
       <c r="D3" s="7">
@@ -4011,52 +4038,484 @@
         <v>58.02</v>
       </c>
     </row>
-    <row r="65" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A65" s="18"/>
-    </row>
-    <row r="66" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A66" s="18"/>
-    </row>
-    <row r="67" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A67" s="18"/>
-    </row>
-    <row r="68" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A68" s="18"/>
-    </row>
-    <row r="69" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A69" s="18"/>
-    </row>
-    <row r="70" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A70" s="18"/>
-    </row>
-    <row r="71" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A71" s="18"/>
-    </row>
-    <row r="72" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A72" s="18"/>
-    </row>
-    <row r="73" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A73" s="18"/>
-    </row>
-    <row r="74" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:16" ht="16" x14ac:dyDescent="0.2">
+      <c r="A65" s="17" t="s">
+        <v>42</v>
+      </c>
+      <c r="B65" t="s">
+        <v>14</v>
+      </c>
+      <c r="C65" s="9">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="D65">
+        <v>0.64739999999999998</v>
+      </c>
+      <c r="E65">
+        <v>0.16600000000000001</v>
+      </c>
+      <c r="F65">
+        <v>0.41220000000000001</v>
+      </c>
+      <c r="G65">
+        <v>7.3899999999999993E-2</v>
+      </c>
+      <c r="H65">
+        <v>0.6966</v>
+      </c>
+      <c r="I65">
+        <v>0.13120000000000001</v>
+      </c>
+      <c r="J65">
+        <v>0.53879999999999995</v>
+      </c>
+      <c r="K65">
+        <v>0.18509999999999999</v>
+      </c>
+      <c r="L65">
+        <v>9.8268000000000004</v>
+      </c>
+      <c r="M65">
+        <v>2.1303000000000001</v>
+      </c>
+      <c r="N65">
+        <v>46.45</v>
+      </c>
+      <c r="O65">
+        <v>20.23</v>
+      </c>
+      <c r="P65">
+        <v>33.32</v>
+      </c>
+    </row>
+    <row r="66" spans="1:16" ht="16" x14ac:dyDescent="0.2">
+      <c r="A66" s="17" t="s">
+        <v>43</v>
+      </c>
+      <c r="B66" t="s">
+        <v>20</v>
+      </c>
+      <c r="C66" s="9">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="D66">
+        <v>0.64739999999999998</v>
+      </c>
+      <c r="E66">
+        <v>0.12859999999999999</v>
+      </c>
+      <c r="F66">
+        <v>0.41620000000000001</v>
+      </c>
+      <c r="G66">
+        <v>2.0299999999999999E-2</v>
+      </c>
+      <c r="H66">
+        <v>0.70660000000000001</v>
+      </c>
+      <c r="I66">
+        <v>0.1477</v>
+      </c>
+      <c r="J66">
+        <v>0.65549999999999997</v>
+      </c>
+      <c r="K66">
+        <v>0.41699999999999998</v>
+      </c>
+      <c r="L66">
+        <v>10.052</v>
+      </c>
+      <c r="M66">
+        <v>2.0897999999999999</v>
+      </c>
+      <c r="N66">
+        <v>31.08</v>
+      </c>
+      <c r="O66">
+        <v>25.36</v>
+      </c>
+      <c r="P66">
+        <v>43.57</v>
+      </c>
+    </row>
+    <row r="67" spans="1:16" ht="16" x14ac:dyDescent="0.2">
+      <c r="A67" s="17" t="s">
+        <v>44</v>
+      </c>
+      <c r="B67" t="s">
+        <v>20</v>
+      </c>
+      <c r="C67" s="9">
+        <f t="shared" ref="C67:C73" si="1">IF(B67="Binder", 1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="D67">
+        <v>0.41270000000000001</v>
+      </c>
+      <c r="E67">
+        <v>8.6099999999999996E-2</v>
+      </c>
+      <c r="F67">
+        <v>0.29199999999999998</v>
+      </c>
+      <c r="G67">
+        <v>3.8300000000000001E-2</v>
+      </c>
+      <c r="H67">
+        <v>0.59160000000000001</v>
+      </c>
+      <c r="I67">
+        <v>0.1295</v>
+      </c>
+      <c r="J67">
+        <v>0.54830000000000001</v>
+      </c>
+      <c r="K67">
+        <v>0.13950000000000001</v>
+      </c>
+      <c r="L67">
+        <v>8.0274999999999999</v>
+      </c>
+      <c r="M67">
+        <v>2.4157000000000002</v>
+      </c>
+      <c r="N67">
+        <v>69.06</v>
+      </c>
+      <c r="O67">
+        <v>12.25</v>
+      </c>
+      <c r="P67">
+        <v>18.68</v>
+      </c>
+    </row>
+    <row r="68" spans="1:16" ht="16" x14ac:dyDescent="0.2">
+      <c r="A68" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="B68" t="s">
+        <v>20</v>
+      </c>
+      <c r="C68" s="9">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="D68">
+        <v>0.36709999999999998</v>
+      </c>
+      <c r="E68">
+        <v>6.8699999999999997E-2</v>
+      </c>
+      <c r="F68">
+        <v>0.45200000000000001</v>
+      </c>
+      <c r="G68">
+        <v>0.16</v>
+      </c>
+      <c r="H68">
+        <v>0.70720000000000005</v>
+      </c>
+      <c r="I68">
+        <v>0.1396</v>
+      </c>
+      <c r="J68">
+        <v>0.62460000000000004</v>
+      </c>
+      <c r="K68">
+        <v>0.18770000000000001</v>
+      </c>
+      <c r="L68">
+        <v>10.586</v>
+      </c>
+      <c r="M68">
+        <v>1.1316999999999999</v>
+      </c>
+      <c r="N68">
+        <v>13.84</v>
+      </c>
+      <c r="O68">
+        <v>20.83</v>
+      </c>
+      <c r="P68">
+        <v>65.34</v>
+      </c>
+    </row>
+    <row r="69" spans="1:16" ht="16" x14ac:dyDescent="0.2">
+      <c r="A69" s="17" t="s">
+        <v>46</v>
+      </c>
+      <c r="B69" t="s">
+        <v>20</v>
+      </c>
+      <c r="C69" s="9">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="D69">
+        <v>0.40789999999999998</v>
+      </c>
+      <c r="E69">
+        <v>9.01E-2</v>
+      </c>
+      <c r="F69">
+        <v>0.88060000000000005</v>
+      </c>
+      <c r="G69">
+        <v>0.1081</v>
+      </c>
+      <c r="H69">
+        <v>0.74819999999999998</v>
+      </c>
+      <c r="I69">
+        <v>0.1187</v>
+      </c>
+      <c r="J69">
+        <v>0.60040000000000004</v>
+      </c>
+      <c r="K69">
+        <v>0.22289999999999999</v>
+      </c>
+      <c r="L69">
+        <v>12.3896</v>
+      </c>
+      <c r="M69">
+        <v>2.0489000000000002</v>
+      </c>
+      <c r="N69">
+        <v>12.69</v>
+      </c>
+      <c r="O69">
+        <v>70.040000000000006</v>
+      </c>
+      <c r="P69">
+        <v>17.27</v>
+      </c>
+    </row>
+    <row r="70" spans="1:16" ht="16" x14ac:dyDescent="0.2">
+      <c r="A70" s="17" t="s">
+        <v>47</v>
+      </c>
+      <c r="B70" t="s">
+        <v>22</v>
+      </c>
+      <c r="C70" s="9">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="D70">
+        <v>0.31869999999999998</v>
+      </c>
+      <c r="E70">
+        <v>5.8900000000000001E-2</v>
+      </c>
+      <c r="F70">
+        <v>0.35420000000000001</v>
+      </c>
+      <c r="G70">
+        <v>8.8300000000000003E-2</v>
+      </c>
+      <c r="H70">
+        <v>0.72719999999999996</v>
+      </c>
+      <c r="I70">
+        <v>0.16200000000000001</v>
+      </c>
+      <c r="J70">
+        <v>0.50070000000000003</v>
+      </c>
+      <c r="K70">
+        <v>0.16439999999999999</v>
+      </c>
+      <c r="L70">
+        <v>10.3277</v>
+      </c>
+      <c r="M70">
+        <v>1.1355</v>
+      </c>
+      <c r="N70">
+        <v>19.75</v>
+      </c>
+      <c r="O70">
+        <v>12.87</v>
+      </c>
+      <c r="P70">
+        <v>67.38</v>
+      </c>
+    </row>
+    <row r="71" spans="1:16" ht="16" x14ac:dyDescent="0.2">
+      <c r="A71" s="17" t="s">
+        <v>48</v>
+      </c>
+      <c r="B71" t="s">
+        <v>22</v>
+      </c>
+      <c r="C71" s="9">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="D71">
+        <v>0.47160000000000002</v>
+      </c>
+      <c r="E71">
+        <v>0.1159</v>
+      </c>
+      <c r="F71">
+        <v>0.3866</v>
+      </c>
+      <c r="G71">
+        <v>5.7799999999999997E-2</v>
+      </c>
+      <c r="H71">
+        <v>0.50829999999999997</v>
+      </c>
+      <c r="I71">
+        <v>8.9899999999999994E-2</v>
+      </c>
+      <c r="J71">
+        <v>0.3049</v>
+      </c>
+      <c r="K71">
+        <v>5.9400000000000001E-2</v>
+      </c>
+      <c r="L71">
+        <v>8.9847000000000001</v>
+      </c>
+      <c r="M71">
+        <v>1.1616</v>
+      </c>
+      <c r="N71">
+        <v>63.18</v>
+      </c>
+      <c r="O71">
+        <v>1.17</v>
+      </c>
+      <c r="P71">
+        <v>35.65</v>
+      </c>
+    </row>
+    <row r="72" spans="1:16" ht="16" x14ac:dyDescent="0.2">
+      <c r="A72" s="17" t="s">
+        <v>49</v>
+      </c>
+      <c r="B72" t="s">
+        <v>22</v>
+      </c>
+      <c r="C72" s="9">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="D72">
+        <v>0.4531</v>
+      </c>
+      <c r="E72">
+        <v>9.8000000000000004E-2</v>
+      </c>
+      <c r="F72">
+        <v>0.98860000000000003</v>
+      </c>
+      <c r="G72">
+        <v>0.46089999999999998</v>
+      </c>
+      <c r="H72">
+        <v>0.61040000000000005</v>
+      </c>
+      <c r="I72">
+        <v>0.1298</v>
+      </c>
+      <c r="J72">
+        <v>0.36449999999999999</v>
+      </c>
+      <c r="K72">
+        <v>8.4400000000000003E-2</v>
+      </c>
+      <c r="L72">
+        <v>11.638500000000001</v>
+      </c>
+      <c r="M72">
+        <v>1.6237999999999999</v>
+      </c>
+      <c r="N72">
+        <v>10.29</v>
+      </c>
+      <c r="O72">
+        <v>48.06</v>
+      </c>
+      <c r="P72">
+        <v>41.65</v>
+      </c>
+    </row>
+    <row r="73" spans="1:16" ht="16" x14ac:dyDescent="0.2">
+      <c r="A73" s="17" t="s">
+        <v>50</v>
+      </c>
+      <c r="B73" t="s">
+        <v>22</v>
+      </c>
+      <c r="C73" s="9">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="D73">
+        <v>0.32329999999999998</v>
+      </c>
+      <c r="E73">
+        <v>5.3999999999999999E-2</v>
+      </c>
+      <c r="F73">
+        <v>0.33300000000000002</v>
+      </c>
+      <c r="G73">
+        <v>7.0300000000000001E-2</v>
+      </c>
+      <c r="H73">
+        <v>0.76539999999999997</v>
+      </c>
+      <c r="I73">
+        <v>0.15</v>
+      </c>
+      <c r="J73">
+        <v>0.66120000000000001</v>
+      </c>
+      <c r="K73">
+        <v>0.20180000000000001</v>
+      </c>
+      <c r="L73">
+        <v>9.0381999999999998</v>
+      </c>
+      <c r="M73">
+        <v>1.1535</v>
+      </c>
+      <c r="N73">
+        <v>69.03</v>
+      </c>
+      <c r="O73">
+        <v>1.8</v>
+      </c>
+      <c r="P73">
+        <v>29.17</v>
+      </c>
+    </row>
+    <row r="74" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A74" s="18"/>
     </row>
-    <row r="75" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A75" s="18"/>
     </row>
-    <row r="76" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A76" s="18"/>
     </row>
-    <row r="77" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A77" s="18"/>
     </row>
-    <row r="78" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A78" s="18"/>
     </row>
-    <row r="79" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A79" s="18"/>
     </row>
-    <row r="80" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A80" s="18"/>
     </row>
     <row r="81" spans="1:1" x14ac:dyDescent="0.2">
@@ -4064,15 +4523,6 @@
     </row>
     <row r="82" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A82" s="18"/>
-    </row>
-    <row r="83" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A83" s="18"/>
-    </row>
-    <row r="84" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A84" s="18"/>
-    </row>
-    <row r="85" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A85" s="18"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:P34" xr:uid="{5E67669D-DCA0-184E-97A6-09176FE4B22E}"/>
@@ -4083,7 +4533,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9885BA85-965B-6440-A501-864EAA87A82C}">
-  <dimension ref="A1:I64"/>
+  <dimension ref="A1:I73"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="4" max="4" width="13.83203125" bestFit="1" customWidth="1"/>
@@ -4161,7 +4611,7 @@
         <v>1</v>
       </c>
       <c r="C3" s="7">
-        <f t="shared" ref="C3:C64" si="0">IF(B3="Binder", 1,0)</f>
+        <f t="shared" ref="C3:C66" si="0">IF(B3="Binder", 1,0)</f>
         <v>1</v>
       </c>
       <c r="D3" s="7">
@@ -6011,6 +6461,276 @@
       </c>
       <c r="I64">
         <v>58.02</v>
+      </c>
+    </row>
+    <row r="65" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A65" s="17" t="s">
+        <v>42</v>
+      </c>
+      <c r="B65" t="s">
+        <v>14</v>
+      </c>
+      <c r="C65" s="9">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="D65">
+        <v>0.64739999999999998</v>
+      </c>
+      <c r="E65">
+        <v>0.41220000000000001</v>
+      </c>
+      <c r="F65">
+        <v>9.8268000000000004</v>
+      </c>
+      <c r="G65">
+        <v>46.45</v>
+      </c>
+      <c r="H65">
+        <v>20.23</v>
+      </c>
+      <c r="I65">
+        <v>33.32</v>
+      </c>
+    </row>
+    <row r="66" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A66" s="17" t="s">
+        <v>43</v>
+      </c>
+      <c r="B66" t="s">
+        <v>20</v>
+      </c>
+      <c r="C66" s="9">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="D66">
+        <v>0.64739999999999998</v>
+      </c>
+      <c r="E66">
+        <v>0.41620000000000001</v>
+      </c>
+      <c r="F66">
+        <v>10.052</v>
+      </c>
+      <c r="G66">
+        <v>31.08</v>
+      </c>
+      <c r="H66">
+        <v>25.36</v>
+      </c>
+      <c r="I66">
+        <v>43.57</v>
+      </c>
+    </row>
+    <row r="67" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A67" s="17" t="s">
+        <v>44</v>
+      </c>
+      <c r="B67" t="s">
+        <v>20</v>
+      </c>
+      <c r="C67" s="9">
+        <f t="shared" ref="C67:C73" si="1">IF(B67="Binder", 1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="D67">
+        <v>0.41270000000000001</v>
+      </c>
+      <c r="E67">
+        <v>0.29199999999999998</v>
+      </c>
+      <c r="F67">
+        <v>8.0274999999999999</v>
+      </c>
+      <c r="G67">
+        <v>69.06</v>
+      </c>
+      <c r="H67">
+        <v>12.25</v>
+      </c>
+      <c r="I67">
+        <v>18.68</v>
+      </c>
+    </row>
+    <row r="68" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A68" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="B68" t="s">
+        <v>20</v>
+      </c>
+      <c r="C68" s="9">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="D68">
+        <v>0.36709999999999998</v>
+      </c>
+      <c r="E68">
+        <v>0.45200000000000001</v>
+      </c>
+      <c r="F68">
+        <v>10.586</v>
+      </c>
+      <c r="G68">
+        <v>13.84</v>
+      </c>
+      <c r="H68">
+        <v>20.83</v>
+      </c>
+      <c r="I68">
+        <v>65.34</v>
+      </c>
+    </row>
+    <row r="69" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A69" s="17" t="s">
+        <v>46</v>
+      </c>
+      <c r="B69" t="s">
+        <v>20</v>
+      </c>
+      <c r="C69" s="9">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="D69">
+        <v>0.40789999999999998</v>
+      </c>
+      <c r="E69">
+        <v>0.88060000000000005</v>
+      </c>
+      <c r="F69">
+        <v>12.3896</v>
+      </c>
+      <c r="G69">
+        <v>12.69</v>
+      </c>
+      <c r="H69">
+        <v>70.040000000000006</v>
+      </c>
+      <c r="I69">
+        <v>17.27</v>
+      </c>
+    </row>
+    <row r="70" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A70" s="17" t="s">
+        <v>47</v>
+      </c>
+      <c r="B70" t="s">
+        <v>22</v>
+      </c>
+      <c r="C70" s="9">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="D70">
+        <v>0.31869999999999998</v>
+      </c>
+      <c r="E70">
+        <v>0.35420000000000001</v>
+      </c>
+      <c r="F70">
+        <v>10.3277</v>
+      </c>
+      <c r="G70">
+        <v>19.75</v>
+      </c>
+      <c r="H70">
+        <v>12.87</v>
+      </c>
+      <c r="I70">
+        <v>67.38</v>
+      </c>
+    </row>
+    <row r="71" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A71" s="17" t="s">
+        <v>48</v>
+      </c>
+      <c r="B71" t="s">
+        <v>22</v>
+      </c>
+      <c r="C71" s="9">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="D71">
+        <v>0.47160000000000002</v>
+      </c>
+      <c r="E71">
+        <v>0.3866</v>
+      </c>
+      <c r="F71">
+        <v>8.9847000000000001</v>
+      </c>
+      <c r="G71">
+        <v>63.18</v>
+      </c>
+      <c r="H71">
+        <v>1.17</v>
+      </c>
+      <c r="I71">
+        <v>35.65</v>
+      </c>
+    </row>
+    <row r="72" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A72" s="17" t="s">
+        <v>49</v>
+      </c>
+      <c r="B72" t="s">
+        <v>22</v>
+      </c>
+      <c r="C72" s="9">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="D72">
+        <v>0.4531</v>
+      </c>
+      <c r="E72">
+        <v>0.98860000000000003</v>
+      </c>
+      <c r="F72">
+        <v>11.638500000000001</v>
+      </c>
+      <c r="G72">
+        <v>10.29</v>
+      </c>
+      <c r="H72">
+        <v>48.06</v>
+      </c>
+      <c r="I72">
+        <v>41.65</v>
+      </c>
+    </row>
+    <row r="73" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A73" s="17" t="s">
+        <v>50</v>
+      </c>
+      <c r="B73" t="s">
+        <v>22</v>
+      </c>
+      <c r="C73" s="9">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="D73">
+        <v>0.32329999999999998</v>
+      </c>
+      <c r="E73">
+        <v>0.33300000000000002</v>
+      </c>
+      <c r="F73">
+        <v>9.0381999999999998</v>
+      </c>
+      <c r="G73">
+        <v>69.03</v>
+      </c>
+      <c r="H73">
+        <v>1.8</v>
+      </c>
+      <c r="I73">
+        <v>29.17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>